<commit_message>
add goles vs Elite
</commit_message>
<xml_diff>
--- a/events.xlsx
+++ b/events.xlsx
@@ -9,14 +9,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="Ah+6QbZHSCvzlfR+OrztUZG/vsSpuk7hjO7EDNb3u+E="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="TmjwHBOzu1jj8/XdnhHSSxNBnDLhYuS/RBD41+S2zdg="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4665" uniqueCount="1588">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4724" uniqueCount="1615">
   <si>
     <t>Event</t>
   </si>
@@ -4780,13 +4780,94 @@
   </si>
   <si>
     <t>89:46</t>
+  </si>
+  <si>
+    <t>ABP a favor</t>
+  </si>
+  <si>
+    <t>14:05</t>
+  </si>
+  <si>
+    <t>14:17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">70;82 </t>
+  </si>
+  <si>
+    <t>Tiro libre</t>
+  </si>
+  <si>
+    <t>Ocasión</t>
+  </si>
+  <si>
+    <t>Elite Sport</t>
+  </si>
+  <si>
+    <t>https://youtu.be/tYhPg3wKq_c</t>
+  </si>
+  <si>
+    <t>GOL</t>
+  </si>
+  <si>
+    <t>Tran. Defensa-Ataque</t>
+  </si>
+  <si>
+    <t>27:08</t>
+  </si>
+  <si>
+    <t>27:23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">32;32 </t>
+  </si>
+  <si>
+    <t>Contra-ataque</t>
+  </si>
+  <si>
+    <t>Progresión</t>
+  </si>
+  <si>
+    <t>28:48</t>
+  </si>
+  <si>
+    <t>29:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">89;50 </t>
+  </si>
+  <si>
+    <t>Penal</t>
+  </si>
+  <si>
+    <t>67:52</t>
+  </si>
+  <si>
+    <t>68:06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">74;58 </t>
+  </si>
+  <si>
+    <t>Tran. Ataque-Defensa</t>
+  </si>
+  <si>
+    <t>85:56</t>
+  </si>
+  <si>
+    <t xml:space="preserve">40;70 </t>
+  </si>
+  <si>
+    <t>Repliegue</t>
+  </si>
+  <si>
+    <t>Ocasión rival</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -4827,6 +4908,15 @@
       <sz val="10.0"/>
       <color theme="10"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
     </font>
   </fonts>
   <fills count="4">
@@ -4939,7 +5029,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="37">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -5003,6 +5093,28 @@
       <alignment shrinkToFit="0" wrapText="0"/>
     </xf>
     <xf borderId="6" fillId="3" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -5051,7 +5163,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:O442" displayName="Table_1" name="Table_1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:O542" displayName="Table_1" name="Table_1" id="1">
   <tableColumns count="15">
     <tableColumn name="Event" id="1"/>
     <tableColumn name="start_time" id="2"/>
@@ -22497,6 +22609,1834 @@
       <c r="O442" s="8" t="s">
         <v>53</v>
       </c>
+    </row>
+    <row r="443" ht="12.75" customHeight="1">
+      <c r="A443" s="29" t="s">
+        <v>1588</v>
+      </c>
+      <c r="B443" s="30" t="s">
+        <v>1589</v>
+      </c>
+      <c r="C443" s="30" t="s">
+        <v>1589</v>
+      </c>
+      <c r="D443" s="30" t="s">
+        <v>1590</v>
+      </c>
+      <c r="E443" s="29" t="s">
+        <v>1591</v>
+      </c>
+      <c r="F443" s="29" t="s">
+        <v>1592</v>
+      </c>
+      <c r="G443" s="29" t="s">
+        <v>1593</v>
+      </c>
+      <c r="H443" s="31" t="s">
+        <v>1594</v>
+      </c>
+      <c r="I443" s="32" t="s">
+        <v>1595</v>
+      </c>
+      <c r="J443" s="22"/>
+      <c r="K443" s="22"/>
+      <c r="L443" s="33" t="s">
+        <v>1596</v>
+      </c>
+      <c r="M443" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="N443" s="8" t="b">
+        <v>0</v>
+      </c>
+      <c r="O443" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="444" ht="12.75" customHeight="1">
+      <c r="A444" s="29" t="s">
+        <v>1597</v>
+      </c>
+      <c r="B444" s="30" t="s">
+        <v>1598</v>
+      </c>
+      <c r="C444" s="30" t="s">
+        <v>1598</v>
+      </c>
+      <c r="D444" s="30" t="s">
+        <v>1599</v>
+      </c>
+      <c r="E444" s="29" t="s">
+        <v>1600</v>
+      </c>
+      <c r="F444" s="29" t="s">
+        <v>1601</v>
+      </c>
+      <c r="G444" s="29" t="s">
+        <v>1602</v>
+      </c>
+      <c r="H444" s="31" t="s">
+        <v>1594</v>
+      </c>
+      <c r="I444" s="32" t="s">
+        <v>1595</v>
+      </c>
+      <c r="J444" s="22"/>
+      <c r="K444" s="22"/>
+      <c r="L444" s="33"/>
+      <c r="M444" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="N444" s="8" t="b">
+        <v>0</v>
+      </c>
+      <c r="O444" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="445" ht="12.75" customHeight="1">
+      <c r="A445" s="29" t="s">
+        <v>1588</v>
+      </c>
+      <c r="B445" s="30" t="s">
+        <v>1603</v>
+      </c>
+      <c r="C445" s="30" t="s">
+        <v>1603</v>
+      </c>
+      <c r="D445" s="30" t="s">
+        <v>1604</v>
+      </c>
+      <c r="E445" s="29" t="s">
+        <v>1605</v>
+      </c>
+      <c r="F445" s="29" t="s">
+        <v>1606</v>
+      </c>
+      <c r="G445" s="29" t="s">
+        <v>1593</v>
+      </c>
+      <c r="H445" s="31" t="s">
+        <v>1594</v>
+      </c>
+      <c r="I445" s="32" t="s">
+        <v>1595</v>
+      </c>
+      <c r="J445" s="22"/>
+      <c r="K445" s="22"/>
+      <c r="L445" s="33" t="s">
+        <v>1596</v>
+      </c>
+      <c r="M445" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="N445" s="8" t="b">
+        <v>0</v>
+      </c>
+      <c r="O445" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="446" ht="12.75" customHeight="1">
+      <c r="A446" s="29" t="s">
+        <v>1597</v>
+      </c>
+      <c r="B446" s="30" t="s">
+        <v>1607</v>
+      </c>
+      <c r="C446" s="30" t="s">
+        <v>1607</v>
+      </c>
+      <c r="D446" s="30" t="s">
+        <v>1608</v>
+      </c>
+      <c r="E446" s="29" t="s">
+        <v>1609</v>
+      </c>
+      <c r="F446" s="29" t="s">
+        <v>1601</v>
+      </c>
+      <c r="G446" s="29" t="s">
+        <v>1593</v>
+      </c>
+      <c r="H446" s="31" t="s">
+        <v>1594</v>
+      </c>
+      <c r="I446" s="32" t="s">
+        <v>1595</v>
+      </c>
+      <c r="J446" s="22"/>
+      <c r="K446" s="22"/>
+      <c r="L446" s="33" t="s">
+        <v>1596</v>
+      </c>
+      <c r="M446" s="8" t="s">
+        <v>919</v>
+      </c>
+      <c r="N446" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="O446" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="447" ht="12.75" customHeight="1">
+      <c r="A447" s="29" t="s">
+        <v>1610</v>
+      </c>
+      <c r="B447" s="30" t="s">
+        <v>1527</v>
+      </c>
+      <c r="C447" s="30" t="s">
+        <v>1527</v>
+      </c>
+      <c r="D447" s="30" t="s">
+        <v>1611</v>
+      </c>
+      <c r="E447" s="29" t="s">
+        <v>1612</v>
+      </c>
+      <c r="F447" s="29" t="s">
+        <v>1613</v>
+      </c>
+      <c r="G447" s="29" t="s">
+        <v>1614</v>
+      </c>
+      <c r="H447" s="31" t="s">
+        <v>1594</v>
+      </c>
+      <c r="I447" s="32" t="s">
+        <v>1595</v>
+      </c>
+      <c r="J447" s="22"/>
+      <c r="K447" s="22"/>
+      <c r="L447" s="33" t="s">
+        <v>1596</v>
+      </c>
+      <c r="M447" s="8" t="s">
+        <v>919</v>
+      </c>
+      <c r="N447" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="O447" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="448" ht="12.75" customHeight="1">
+      <c r="A448" s="34"/>
+      <c r="B448" s="35"/>
+      <c r="C448" s="35"/>
+      <c r="D448" s="35"/>
+      <c r="E448" s="36"/>
+      <c r="F448" s="36"/>
+      <c r="G448" s="36"/>
+      <c r="H448" s="8"/>
+      <c r="I448" s="9"/>
+      <c r="J448" s="22"/>
+      <c r="K448" s="22"/>
+      <c r="L448" s="36"/>
+      <c r="M448" s="8"/>
+      <c r="N448" s="8"/>
+      <c r="O448" s="8"/>
+    </row>
+    <row r="449" ht="12.75" customHeight="1">
+      <c r="A449" s="34"/>
+      <c r="B449" s="35"/>
+      <c r="C449" s="35"/>
+      <c r="D449" s="35"/>
+      <c r="E449" s="36"/>
+      <c r="F449" s="36"/>
+      <c r="G449" s="36"/>
+      <c r="H449" s="8"/>
+      <c r="I449" s="9"/>
+      <c r="J449" s="22"/>
+      <c r="K449" s="22"/>
+      <c r="L449" s="36"/>
+      <c r="M449" s="8"/>
+      <c r="N449" s="8"/>
+      <c r="O449" s="8"/>
+    </row>
+    <row r="450" ht="12.75" customHeight="1">
+      <c r="A450" s="34"/>
+      <c r="B450" s="35"/>
+      <c r="C450" s="35"/>
+      <c r="D450" s="35"/>
+      <c r="E450" s="36"/>
+      <c r="F450" s="36"/>
+      <c r="G450" s="36"/>
+      <c r="H450" s="8"/>
+      <c r="I450" s="9"/>
+      <c r="J450" s="22"/>
+      <c r="K450" s="22"/>
+      <c r="L450" s="36"/>
+      <c r="M450" s="8"/>
+      <c r="N450" s="8"/>
+      <c r="O450" s="8"/>
+    </row>
+    <row r="451" ht="12.75" customHeight="1">
+      <c r="A451" s="34"/>
+      <c r="B451" s="35"/>
+      <c r="C451" s="35"/>
+      <c r="D451" s="35"/>
+      <c r="E451" s="36"/>
+      <c r="F451" s="36"/>
+      <c r="G451" s="36"/>
+      <c r="H451" s="8"/>
+      <c r="I451" s="9"/>
+      <c r="J451" s="22"/>
+      <c r="K451" s="22"/>
+      <c r="L451" s="36"/>
+      <c r="M451" s="8"/>
+      <c r="N451" s="8"/>
+      <c r="O451" s="8"/>
+    </row>
+    <row r="452" ht="12.75" customHeight="1">
+      <c r="A452" s="34"/>
+      <c r="B452" s="35"/>
+      <c r="C452" s="35"/>
+      <c r="D452" s="35"/>
+      <c r="E452" s="36"/>
+      <c r="F452" s="36"/>
+      <c r="G452" s="36"/>
+      <c r="H452" s="8"/>
+      <c r="I452" s="9"/>
+      <c r="J452" s="22"/>
+      <c r="K452" s="22"/>
+      <c r="L452" s="36"/>
+      <c r="M452" s="8"/>
+      <c r="N452" s="8"/>
+      <c r="O452" s="8"/>
+    </row>
+    <row r="453" ht="12.75" customHeight="1">
+      <c r="A453" s="34"/>
+      <c r="B453" s="35"/>
+      <c r="C453" s="35"/>
+      <c r="D453" s="35"/>
+      <c r="E453" s="36"/>
+      <c r="F453" s="36"/>
+      <c r="G453" s="36"/>
+      <c r="H453" s="8"/>
+      <c r="I453" s="9"/>
+      <c r="J453" s="22"/>
+      <c r="K453" s="22"/>
+      <c r="L453" s="36"/>
+      <c r="M453" s="8"/>
+      <c r="N453" s="8"/>
+      <c r="O453" s="8"/>
+    </row>
+    <row r="454" ht="12.75" customHeight="1">
+      <c r="A454" s="34"/>
+      <c r="B454" s="35"/>
+      <c r="C454" s="35"/>
+      <c r="D454" s="35"/>
+      <c r="E454" s="36"/>
+      <c r="F454" s="36"/>
+      <c r="G454" s="36"/>
+      <c r="H454" s="8"/>
+      <c r="I454" s="9"/>
+      <c r="J454" s="22"/>
+      <c r="K454" s="22"/>
+      <c r="L454" s="36"/>
+      <c r="M454" s="8"/>
+      <c r="N454" s="8"/>
+      <c r="O454" s="8"/>
+    </row>
+    <row r="455" ht="12.75" customHeight="1">
+      <c r="A455" s="34"/>
+      <c r="B455" s="35"/>
+      <c r="C455" s="35"/>
+      <c r="D455" s="35"/>
+      <c r="E455" s="36"/>
+      <c r="F455" s="36"/>
+      <c r="G455" s="36"/>
+      <c r="H455" s="8"/>
+      <c r="I455" s="9"/>
+      <c r="J455" s="22"/>
+      <c r="K455" s="22"/>
+      <c r="L455" s="36"/>
+      <c r="M455" s="8"/>
+      <c r="N455" s="8"/>
+      <c r="O455" s="8"/>
+    </row>
+    <row r="456" ht="12.75" customHeight="1">
+      <c r="A456" s="34"/>
+      <c r="B456" s="35"/>
+      <c r="C456" s="35"/>
+      <c r="D456" s="35"/>
+      <c r="E456" s="36"/>
+      <c r="F456" s="36"/>
+      <c r="G456" s="36"/>
+      <c r="H456" s="8"/>
+      <c r="I456" s="9"/>
+      <c r="J456" s="22"/>
+      <c r="K456" s="22"/>
+      <c r="L456" s="36"/>
+      <c r="M456" s="8"/>
+      <c r="N456" s="8"/>
+      <c r="O456" s="8"/>
+    </row>
+    <row r="457" ht="12.75" customHeight="1">
+      <c r="A457" s="34"/>
+      <c r="B457" s="35"/>
+      <c r="C457" s="35"/>
+      <c r="D457" s="35"/>
+      <c r="E457" s="36"/>
+      <c r="F457" s="36"/>
+      <c r="G457" s="36"/>
+      <c r="H457" s="8"/>
+      <c r="I457" s="9"/>
+      <c r="J457" s="22"/>
+      <c r="K457" s="22"/>
+      <c r="L457" s="36"/>
+      <c r="M457" s="8"/>
+      <c r="N457" s="8"/>
+      <c r="O457" s="8"/>
+    </row>
+    <row r="458" ht="12.75" customHeight="1">
+      <c r="A458" s="34"/>
+      <c r="B458" s="35"/>
+      <c r="C458" s="35"/>
+      <c r="D458" s="35"/>
+      <c r="E458" s="36"/>
+      <c r="F458" s="36"/>
+      <c r="G458" s="36"/>
+      <c r="H458" s="8"/>
+      <c r="I458" s="9"/>
+      <c r="J458" s="22"/>
+      <c r="K458" s="22"/>
+      <c r="L458" s="36"/>
+      <c r="M458" s="8"/>
+      <c r="N458" s="8"/>
+      <c r="O458" s="8"/>
+    </row>
+    <row r="459" ht="12.75" customHeight="1">
+      <c r="A459" s="34"/>
+      <c r="B459" s="35"/>
+      <c r="C459" s="35"/>
+      <c r="D459" s="35"/>
+      <c r="E459" s="36"/>
+      <c r="F459" s="36"/>
+      <c r="G459" s="36"/>
+      <c r="H459" s="8"/>
+      <c r="I459" s="9"/>
+      <c r="J459" s="22"/>
+      <c r="K459" s="22"/>
+      <c r="L459" s="36"/>
+      <c r="M459" s="8"/>
+      <c r="N459" s="8"/>
+      <c r="O459" s="8"/>
+    </row>
+    <row r="460" ht="12.75" customHeight="1">
+      <c r="A460" s="34"/>
+      <c r="B460" s="35"/>
+      <c r="C460" s="35"/>
+      <c r="D460" s="35"/>
+      <c r="E460" s="36"/>
+      <c r="F460" s="36"/>
+      <c r="G460" s="36"/>
+      <c r="H460" s="8"/>
+      <c r="I460" s="9"/>
+      <c r="J460" s="22"/>
+      <c r="K460" s="22"/>
+      <c r="L460" s="36"/>
+      <c r="M460" s="8"/>
+      <c r="N460" s="8"/>
+      <c r="O460" s="8"/>
+    </row>
+    <row r="461" ht="12.75" customHeight="1">
+      <c r="A461" s="34"/>
+      <c r="B461" s="35"/>
+      <c r="C461" s="35"/>
+      <c r="D461" s="35"/>
+      <c r="E461" s="36"/>
+      <c r="F461" s="36"/>
+      <c r="G461" s="36"/>
+      <c r="H461" s="8"/>
+      <c r="I461" s="9"/>
+      <c r="J461" s="22"/>
+      <c r="K461" s="22"/>
+      <c r="L461" s="36"/>
+      <c r="M461" s="8"/>
+      <c r="N461" s="8"/>
+      <c r="O461" s="8"/>
+    </row>
+    <row r="462" ht="12.75" customHeight="1">
+      <c r="A462" s="34"/>
+      <c r="B462" s="35"/>
+      <c r="C462" s="35"/>
+      <c r="D462" s="35"/>
+      <c r="E462" s="36"/>
+      <c r="F462" s="36"/>
+      <c r="G462" s="36"/>
+      <c r="H462" s="8"/>
+      <c r="I462" s="9"/>
+      <c r="J462" s="22"/>
+      <c r="K462" s="22"/>
+      <c r="L462" s="36"/>
+      <c r="M462" s="8"/>
+      <c r="N462" s="8"/>
+      <c r="O462" s="8"/>
+    </row>
+    <row r="463" ht="12.75" customHeight="1">
+      <c r="A463" s="34"/>
+      <c r="B463" s="35"/>
+      <c r="C463" s="35"/>
+      <c r="D463" s="35"/>
+      <c r="E463" s="36"/>
+      <c r="F463" s="36"/>
+      <c r="G463" s="36"/>
+      <c r="H463" s="8"/>
+      <c r="I463" s="9"/>
+      <c r="J463" s="22"/>
+      <c r="K463" s="22"/>
+      <c r="L463" s="36"/>
+      <c r="M463" s="8"/>
+      <c r="N463" s="8"/>
+      <c r="O463" s="8"/>
+    </row>
+    <row r="464" ht="12.75" customHeight="1">
+      <c r="A464" s="34"/>
+      <c r="B464" s="35"/>
+      <c r="C464" s="35"/>
+      <c r="D464" s="35"/>
+      <c r="E464" s="36"/>
+      <c r="F464" s="36"/>
+      <c r="G464" s="36"/>
+      <c r="H464" s="8"/>
+      <c r="I464" s="9"/>
+      <c r="J464" s="22"/>
+      <c r="K464" s="22"/>
+      <c r="L464" s="36"/>
+      <c r="M464" s="8"/>
+      <c r="N464" s="8"/>
+      <c r="O464" s="8"/>
+    </row>
+    <row r="465" ht="12.75" customHeight="1">
+      <c r="A465" s="34"/>
+      <c r="B465" s="35"/>
+      <c r="C465" s="35"/>
+      <c r="D465" s="35"/>
+      <c r="E465" s="36"/>
+      <c r="F465" s="36"/>
+      <c r="G465" s="36"/>
+      <c r="H465" s="8"/>
+      <c r="I465" s="9"/>
+      <c r="J465" s="22"/>
+      <c r="K465" s="22"/>
+      <c r="L465" s="36"/>
+      <c r="M465" s="8"/>
+      <c r="N465" s="8"/>
+      <c r="O465" s="8"/>
+    </row>
+    <row r="466" ht="12.75" customHeight="1">
+      <c r="A466" s="34"/>
+      <c r="B466" s="35"/>
+      <c r="C466" s="35"/>
+      <c r="D466" s="35"/>
+      <c r="E466" s="36"/>
+      <c r="F466" s="36"/>
+      <c r="G466" s="36"/>
+      <c r="H466" s="8"/>
+      <c r="I466" s="9"/>
+      <c r="J466" s="22"/>
+      <c r="K466" s="22"/>
+      <c r="L466" s="36"/>
+      <c r="M466" s="8"/>
+      <c r="N466" s="8"/>
+      <c r="O466" s="8"/>
+    </row>
+    <row r="467" ht="12.75" customHeight="1">
+      <c r="A467" s="34"/>
+      <c r="B467" s="35"/>
+      <c r="C467" s="35"/>
+      <c r="D467" s="35"/>
+      <c r="E467" s="36"/>
+      <c r="F467" s="36"/>
+      <c r="G467" s="36"/>
+      <c r="H467" s="8"/>
+      <c r="I467" s="9"/>
+      <c r="J467" s="22"/>
+      <c r="K467" s="22"/>
+      <c r="L467" s="36"/>
+      <c r="M467" s="8"/>
+      <c r="N467" s="8"/>
+      <c r="O467" s="8"/>
+    </row>
+    <row r="468" ht="12.75" customHeight="1">
+      <c r="A468" s="34"/>
+      <c r="B468" s="35"/>
+      <c r="C468" s="35"/>
+      <c r="D468" s="35"/>
+      <c r="E468" s="36"/>
+      <c r="F468" s="36"/>
+      <c r="G468" s="36"/>
+      <c r="H468" s="8"/>
+      <c r="I468" s="9"/>
+      <c r="J468" s="22"/>
+      <c r="K468" s="22"/>
+      <c r="L468" s="36"/>
+      <c r="M468" s="8"/>
+      <c r="N468" s="8"/>
+      <c r="O468" s="8"/>
+    </row>
+    <row r="469" ht="12.75" customHeight="1">
+      <c r="A469" s="34"/>
+      <c r="B469" s="35"/>
+      <c r="C469" s="35"/>
+      <c r="D469" s="35"/>
+      <c r="E469" s="36"/>
+      <c r="F469" s="36"/>
+      <c r="G469" s="36"/>
+      <c r="H469" s="8"/>
+      <c r="I469" s="9"/>
+      <c r="J469" s="22"/>
+      <c r="K469" s="22"/>
+      <c r="L469" s="36"/>
+      <c r="M469" s="8"/>
+      <c r="N469" s="8"/>
+      <c r="O469" s="8"/>
+    </row>
+    <row r="470" ht="12.75" customHeight="1">
+      <c r="A470" s="34"/>
+      <c r="B470" s="35"/>
+      <c r="C470" s="35"/>
+      <c r="D470" s="35"/>
+      <c r="E470" s="36"/>
+      <c r="F470" s="36"/>
+      <c r="G470" s="36"/>
+      <c r="H470" s="8"/>
+      <c r="I470" s="9"/>
+      <c r="J470" s="22"/>
+      <c r="K470" s="22"/>
+      <c r="L470" s="36"/>
+      <c r="M470" s="8"/>
+      <c r="N470" s="8"/>
+      <c r="O470" s="8"/>
+    </row>
+    <row r="471" ht="12.75" customHeight="1">
+      <c r="A471" s="34"/>
+      <c r="B471" s="35"/>
+      <c r="C471" s="35"/>
+      <c r="D471" s="35"/>
+      <c r="E471" s="36"/>
+      <c r="F471" s="36"/>
+      <c r="G471" s="36"/>
+      <c r="H471" s="8"/>
+      <c r="I471" s="9"/>
+      <c r="J471" s="22"/>
+      <c r="K471" s="22"/>
+      <c r="L471" s="36"/>
+      <c r="M471" s="8"/>
+      <c r="N471" s="8"/>
+      <c r="O471" s="8"/>
+    </row>
+    <row r="472" ht="12.75" customHeight="1">
+      <c r="A472" s="34"/>
+      <c r="B472" s="35"/>
+      <c r="C472" s="35"/>
+      <c r="D472" s="35"/>
+      <c r="E472" s="36"/>
+      <c r="F472" s="36"/>
+      <c r="G472" s="36"/>
+      <c r="H472" s="8"/>
+      <c r="I472" s="9"/>
+      <c r="J472" s="22"/>
+      <c r="K472" s="22"/>
+      <c r="L472" s="36"/>
+      <c r="M472" s="8"/>
+      <c r="N472" s="8"/>
+      <c r="O472" s="8"/>
+    </row>
+    <row r="473" ht="12.75" customHeight="1">
+      <c r="A473" s="34"/>
+      <c r="B473" s="35"/>
+      <c r="C473" s="35"/>
+      <c r="D473" s="35"/>
+      <c r="E473" s="36"/>
+      <c r="F473" s="36"/>
+      <c r="G473" s="36"/>
+      <c r="H473" s="8"/>
+      <c r="I473" s="9"/>
+      <c r="J473" s="22"/>
+      <c r="K473" s="22"/>
+      <c r="L473" s="36"/>
+      <c r="M473" s="8"/>
+      <c r="N473" s="8"/>
+      <c r="O473" s="8"/>
+    </row>
+    <row r="474" ht="12.75" customHeight="1">
+      <c r="A474" s="34"/>
+      <c r="B474" s="35"/>
+      <c r="C474" s="35"/>
+      <c r="D474" s="35"/>
+      <c r="E474" s="36"/>
+      <c r="F474" s="36"/>
+      <c r="G474" s="36"/>
+      <c r="H474" s="8"/>
+      <c r="I474" s="9"/>
+      <c r="J474" s="22"/>
+      <c r="K474" s="22"/>
+      <c r="L474" s="36"/>
+      <c r="M474" s="8"/>
+      <c r="N474" s="8"/>
+      <c r="O474" s="8"/>
+    </row>
+    <row r="475" ht="12.75" customHeight="1">
+      <c r="A475" s="34"/>
+      <c r="B475" s="35"/>
+      <c r="C475" s="35"/>
+      <c r="D475" s="35"/>
+      <c r="E475" s="36"/>
+      <c r="F475" s="36"/>
+      <c r="G475" s="36"/>
+      <c r="H475" s="8"/>
+      <c r="I475" s="9"/>
+      <c r="J475" s="22"/>
+      <c r="K475" s="22"/>
+      <c r="L475" s="36"/>
+      <c r="M475" s="8"/>
+      <c r="N475" s="8"/>
+      <c r="O475" s="8"/>
+    </row>
+    <row r="476" ht="12.75" customHeight="1">
+      <c r="A476" s="34"/>
+      <c r="B476" s="35"/>
+      <c r="C476" s="35"/>
+      <c r="D476" s="35"/>
+      <c r="E476" s="36"/>
+      <c r="F476" s="36"/>
+      <c r="G476" s="36"/>
+      <c r="H476" s="8"/>
+      <c r="I476" s="9"/>
+      <c r="J476" s="22"/>
+      <c r="K476" s="22"/>
+      <c r="L476" s="36"/>
+      <c r="M476" s="8"/>
+      <c r="N476" s="8"/>
+      <c r="O476" s="8"/>
+    </row>
+    <row r="477" ht="12.75" customHeight="1">
+      <c r="A477" s="34"/>
+      <c r="B477" s="35"/>
+      <c r="C477" s="35"/>
+      <c r="D477" s="35"/>
+      <c r="E477" s="36"/>
+      <c r="F477" s="36"/>
+      <c r="G477" s="36"/>
+      <c r="H477" s="8"/>
+      <c r="I477" s="9"/>
+      <c r="J477" s="22"/>
+      <c r="K477" s="22"/>
+      <c r="L477" s="36"/>
+      <c r="M477" s="8"/>
+      <c r="N477" s="8"/>
+      <c r="O477" s="8"/>
+    </row>
+    <row r="478" ht="12.75" customHeight="1">
+      <c r="A478" s="34"/>
+      <c r="B478" s="35"/>
+      <c r="C478" s="35"/>
+      <c r="D478" s="35"/>
+      <c r="E478" s="36"/>
+      <c r="F478" s="36"/>
+      <c r="G478" s="36"/>
+      <c r="H478" s="8"/>
+      <c r="I478" s="9"/>
+      <c r="J478" s="22"/>
+      <c r="K478" s="22"/>
+      <c r="L478" s="36"/>
+      <c r="M478" s="8"/>
+      <c r="N478" s="8"/>
+      <c r="O478" s="8"/>
+    </row>
+    <row r="479" ht="12.75" customHeight="1">
+      <c r="A479" s="34"/>
+      <c r="B479" s="35"/>
+      <c r="C479" s="35"/>
+      <c r="D479" s="35"/>
+      <c r="E479" s="36"/>
+      <c r="F479" s="36"/>
+      <c r="G479" s="36"/>
+      <c r="H479" s="8"/>
+      <c r="I479" s="9"/>
+      <c r="J479" s="22"/>
+      <c r="K479" s="22"/>
+      <c r="L479" s="36"/>
+      <c r="M479" s="8"/>
+      <c r="N479" s="8"/>
+      <c r="O479" s="8"/>
+    </row>
+    <row r="480" ht="12.75" customHeight="1">
+      <c r="A480" s="34"/>
+      <c r="B480" s="35"/>
+      <c r="C480" s="35"/>
+      <c r="D480" s="35"/>
+      <c r="E480" s="36"/>
+      <c r="F480" s="36"/>
+      <c r="G480" s="36"/>
+      <c r="H480" s="8"/>
+      <c r="I480" s="9"/>
+      <c r="J480" s="22"/>
+      <c r="K480" s="22"/>
+      <c r="L480" s="36"/>
+      <c r="M480" s="8"/>
+      <c r="N480" s="8"/>
+      <c r="O480" s="8"/>
+    </row>
+    <row r="481" ht="12.75" customHeight="1">
+      <c r="A481" s="34"/>
+      <c r="B481" s="35"/>
+      <c r="C481" s="35"/>
+      <c r="D481" s="35"/>
+      <c r="E481" s="36"/>
+      <c r="F481" s="36"/>
+      <c r="G481" s="36"/>
+      <c r="H481" s="8"/>
+      <c r="I481" s="9"/>
+      <c r="J481" s="22"/>
+      <c r="K481" s="22"/>
+      <c r="L481" s="36"/>
+      <c r="M481" s="8"/>
+      <c r="N481" s="8"/>
+      <c r="O481" s="8"/>
+    </row>
+    <row r="482" ht="12.75" customHeight="1">
+      <c r="A482" s="34"/>
+      <c r="B482" s="35"/>
+      <c r="C482" s="35"/>
+      <c r="D482" s="35"/>
+      <c r="E482" s="36"/>
+      <c r="F482" s="36"/>
+      <c r="G482" s="36"/>
+      <c r="H482" s="8"/>
+      <c r="I482" s="9"/>
+      <c r="J482" s="22"/>
+      <c r="K482" s="22"/>
+      <c r="L482" s="36"/>
+      <c r="M482" s="8"/>
+      <c r="N482" s="8"/>
+      <c r="O482" s="8"/>
+    </row>
+    <row r="483" ht="12.75" customHeight="1">
+      <c r="A483" s="34"/>
+      <c r="B483" s="35"/>
+      <c r="C483" s="35"/>
+      <c r="D483" s="35"/>
+      <c r="E483" s="36"/>
+      <c r="F483" s="36"/>
+      <c r="G483" s="36"/>
+      <c r="H483" s="8"/>
+      <c r="I483" s="9"/>
+      <c r="J483" s="22"/>
+      <c r="K483" s="22"/>
+      <c r="L483" s="36"/>
+      <c r="M483" s="8"/>
+      <c r="N483" s="8"/>
+      <c r="O483" s="8"/>
+    </row>
+    <row r="484" ht="12.75" customHeight="1">
+      <c r="A484" s="34"/>
+      <c r="B484" s="35"/>
+      <c r="C484" s="35"/>
+      <c r="D484" s="35"/>
+      <c r="E484" s="36"/>
+      <c r="F484" s="36"/>
+      <c r="G484" s="36"/>
+      <c r="H484" s="8"/>
+      <c r="I484" s="9"/>
+      <c r="J484" s="22"/>
+      <c r="K484" s="22"/>
+      <c r="L484" s="36"/>
+      <c r="M484" s="8"/>
+      <c r="N484" s="8"/>
+      <c r="O484" s="8"/>
+    </row>
+    <row r="485" ht="12.75" customHeight="1">
+      <c r="A485" s="34"/>
+      <c r="B485" s="35"/>
+      <c r="C485" s="35"/>
+      <c r="D485" s="35"/>
+      <c r="E485" s="36"/>
+      <c r="F485" s="36"/>
+      <c r="G485" s="36"/>
+      <c r="H485" s="8"/>
+      <c r="I485" s="9"/>
+      <c r="J485" s="22"/>
+      <c r="K485" s="22"/>
+      <c r="L485" s="36"/>
+      <c r="M485" s="8"/>
+      <c r="N485" s="8"/>
+      <c r="O485" s="8"/>
+    </row>
+    <row r="486" ht="12.75" customHeight="1">
+      <c r="A486" s="34"/>
+      <c r="B486" s="35"/>
+      <c r="C486" s="35"/>
+      <c r="D486" s="35"/>
+      <c r="E486" s="36"/>
+      <c r="F486" s="36"/>
+      <c r="G486" s="36"/>
+      <c r="H486" s="8"/>
+      <c r="I486" s="9"/>
+      <c r="J486" s="22"/>
+      <c r="K486" s="22"/>
+      <c r="L486" s="36"/>
+      <c r="M486" s="8"/>
+      <c r="N486" s="8"/>
+      <c r="O486" s="8"/>
+    </row>
+    <row r="487" ht="12.75" customHeight="1">
+      <c r="A487" s="34"/>
+      <c r="B487" s="35"/>
+      <c r="C487" s="35"/>
+      <c r="D487" s="35"/>
+      <c r="E487" s="36"/>
+      <c r="F487" s="36"/>
+      <c r="G487" s="36"/>
+      <c r="H487" s="8"/>
+      <c r="I487" s="9"/>
+      <c r="J487" s="22"/>
+      <c r="K487" s="22"/>
+      <c r="L487" s="36"/>
+      <c r="M487" s="8"/>
+      <c r="N487" s="8"/>
+      <c r="O487" s="8"/>
+    </row>
+    <row r="488" ht="12.75" customHeight="1">
+      <c r="A488" s="34"/>
+      <c r="B488" s="35"/>
+      <c r="C488" s="35"/>
+      <c r="D488" s="35"/>
+      <c r="E488" s="36"/>
+      <c r="F488" s="36"/>
+      <c r="G488" s="36"/>
+      <c r="H488" s="8"/>
+      <c r="I488" s="9"/>
+      <c r="J488" s="22"/>
+      <c r="K488" s="22"/>
+      <c r="L488" s="36"/>
+      <c r="M488" s="8"/>
+      <c r="N488" s="8"/>
+      <c r="O488" s="8"/>
+    </row>
+    <row r="489" ht="12.75" customHeight="1">
+      <c r="A489" s="34"/>
+      <c r="B489" s="35"/>
+      <c r="C489" s="35"/>
+      <c r="D489" s="35"/>
+      <c r="E489" s="36"/>
+      <c r="F489" s="36"/>
+      <c r="G489" s="36"/>
+      <c r="H489" s="8"/>
+      <c r="I489" s="9"/>
+      <c r="J489" s="22"/>
+      <c r="K489" s="22"/>
+      <c r="L489" s="36"/>
+      <c r="M489" s="8"/>
+      <c r="N489" s="8"/>
+      <c r="O489" s="8"/>
+    </row>
+    <row r="490" ht="12.75" customHeight="1">
+      <c r="A490" s="34"/>
+      <c r="B490" s="35"/>
+      <c r="C490" s="35"/>
+      <c r="D490" s="35"/>
+      <c r="E490" s="36"/>
+      <c r="F490" s="36"/>
+      <c r="G490" s="36"/>
+      <c r="H490" s="8"/>
+      <c r="I490" s="9"/>
+      <c r="J490" s="22"/>
+      <c r="K490" s="22"/>
+      <c r="L490" s="36"/>
+      <c r="M490" s="8"/>
+      <c r="N490" s="8"/>
+      <c r="O490" s="8"/>
+    </row>
+    <row r="491" ht="12.75" customHeight="1">
+      <c r="A491" s="34"/>
+      <c r="B491" s="35"/>
+      <c r="C491" s="35"/>
+      <c r="D491" s="35"/>
+      <c r="E491" s="36"/>
+      <c r="F491" s="36"/>
+      <c r="G491" s="36"/>
+      <c r="H491" s="8"/>
+      <c r="I491" s="9"/>
+      <c r="J491" s="22"/>
+      <c r="K491" s="22"/>
+      <c r="L491" s="36"/>
+      <c r="M491" s="8"/>
+      <c r="N491" s="8"/>
+      <c r="O491" s="8"/>
+    </row>
+    <row r="492" ht="12.75" customHeight="1">
+      <c r="A492" s="34"/>
+      <c r="B492" s="35"/>
+      <c r="C492" s="35"/>
+      <c r="D492" s="35"/>
+      <c r="E492" s="36"/>
+      <c r="F492" s="36"/>
+      <c r="G492" s="36"/>
+      <c r="H492" s="8"/>
+      <c r="I492" s="9"/>
+      <c r="J492" s="22"/>
+      <c r="K492" s="22"/>
+      <c r="L492" s="36"/>
+      <c r="M492" s="8"/>
+      <c r="N492" s="8"/>
+      <c r="O492" s="8"/>
+    </row>
+    <row r="493" ht="12.75" customHeight="1">
+      <c r="A493" s="34"/>
+      <c r="B493" s="35"/>
+      <c r="C493" s="35"/>
+      <c r="D493" s="35"/>
+      <c r="E493" s="36"/>
+      <c r="F493" s="36"/>
+      <c r="G493" s="36"/>
+      <c r="H493" s="8"/>
+      <c r="I493" s="9"/>
+      <c r="J493" s="22"/>
+      <c r="K493" s="22"/>
+      <c r="L493" s="36"/>
+      <c r="M493" s="8"/>
+      <c r="N493" s="8"/>
+      <c r="O493" s="8"/>
+    </row>
+    <row r="494" ht="12.75" customHeight="1">
+      <c r="A494" s="34"/>
+      <c r="B494" s="35"/>
+      <c r="C494" s="35"/>
+      <c r="D494" s="35"/>
+      <c r="E494" s="36"/>
+      <c r="F494" s="36"/>
+      <c r="G494" s="36"/>
+      <c r="H494" s="8"/>
+      <c r="I494" s="9"/>
+      <c r="J494" s="22"/>
+      <c r="K494" s="22"/>
+      <c r="L494" s="36"/>
+      <c r="M494" s="8"/>
+      <c r="N494" s="8"/>
+      <c r="O494" s="8"/>
+    </row>
+    <row r="495" ht="12.75" customHeight="1">
+      <c r="A495" s="34"/>
+      <c r="B495" s="35"/>
+      <c r="C495" s="35"/>
+      <c r="D495" s="35"/>
+      <c r="E495" s="36"/>
+      <c r="F495" s="36"/>
+      <c r="G495" s="36"/>
+      <c r="H495" s="8"/>
+      <c r="I495" s="9"/>
+      <c r="J495" s="22"/>
+      <c r="K495" s="22"/>
+      <c r="L495" s="36"/>
+      <c r="M495" s="8"/>
+      <c r="N495" s="8"/>
+      <c r="O495" s="8"/>
+    </row>
+    <row r="496" ht="12.75" customHeight="1">
+      <c r="A496" s="34"/>
+      <c r="B496" s="35"/>
+      <c r="C496" s="35"/>
+      <c r="D496" s="35"/>
+      <c r="E496" s="36"/>
+      <c r="F496" s="36"/>
+      <c r="G496" s="36"/>
+      <c r="H496" s="8"/>
+      <c r="I496" s="9"/>
+      <c r="J496" s="22"/>
+      <c r="K496" s="22"/>
+      <c r="L496" s="36"/>
+      <c r="M496" s="8"/>
+      <c r="N496" s="8"/>
+      <c r="O496" s="8"/>
+    </row>
+    <row r="497" ht="12.75" customHeight="1">
+      <c r="A497" s="34"/>
+      <c r="B497" s="35"/>
+      <c r="C497" s="35"/>
+      <c r="D497" s="35"/>
+      <c r="E497" s="36"/>
+      <c r="F497" s="36"/>
+      <c r="G497" s="36"/>
+      <c r="H497" s="8"/>
+      <c r="I497" s="9"/>
+      <c r="J497" s="22"/>
+      <c r="K497" s="22"/>
+      <c r="L497" s="36"/>
+      <c r="M497" s="8"/>
+      <c r="N497" s="8"/>
+      <c r="O497" s="8"/>
+    </row>
+    <row r="498" ht="12.75" customHeight="1">
+      <c r="A498" s="34"/>
+      <c r="B498" s="35"/>
+      <c r="C498" s="35"/>
+      <c r="D498" s="35"/>
+      <c r="E498" s="36"/>
+      <c r="F498" s="36"/>
+      <c r="G498" s="36"/>
+      <c r="H498" s="8"/>
+      <c r="I498" s="9"/>
+      <c r="J498" s="22"/>
+      <c r="K498" s="22"/>
+      <c r="L498" s="36"/>
+      <c r="M498" s="8"/>
+      <c r="N498" s="8"/>
+      <c r="O498" s="8"/>
+    </row>
+    <row r="499" ht="12.75" customHeight="1">
+      <c r="A499" s="34"/>
+      <c r="B499" s="35"/>
+      <c r="C499" s="35"/>
+      <c r="D499" s="35"/>
+      <c r="E499" s="36"/>
+      <c r="F499" s="36"/>
+      <c r="G499" s="36"/>
+      <c r="H499" s="8"/>
+      <c r="I499" s="9"/>
+      <c r="J499" s="22"/>
+      <c r="K499" s="22"/>
+      <c r="L499" s="36"/>
+      <c r="M499" s="8"/>
+      <c r="N499" s="8"/>
+      <c r="O499" s="8"/>
+    </row>
+    <row r="500" ht="12.75" customHeight="1">
+      <c r="A500" s="34"/>
+      <c r="B500" s="35"/>
+      <c r="C500" s="35"/>
+      <c r="D500" s="35"/>
+      <c r="E500" s="36"/>
+      <c r="F500" s="36"/>
+      <c r="G500" s="36"/>
+      <c r="H500" s="8"/>
+      <c r="I500" s="9"/>
+      <c r="J500" s="22"/>
+      <c r="K500" s="22"/>
+      <c r="L500" s="36"/>
+      <c r="M500" s="8"/>
+      <c r="N500" s="8"/>
+      <c r="O500" s="8"/>
+    </row>
+    <row r="501" ht="12.75" customHeight="1">
+      <c r="A501" s="34"/>
+      <c r="B501" s="35"/>
+      <c r="C501" s="35"/>
+      <c r="D501" s="35"/>
+      <c r="E501" s="36"/>
+      <c r="F501" s="36"/>
+      <c r="G501" s="36"/>
+      <c r="H501" s="8"/>
+      <c r="I501" s="9"/>
+      <c r="J501" s="22"/>
+      <c r="K501" s="22"/>
+      <c r="L501" s="36"/>
+      <c r="M501" s="8"/>
+      <c r="N501" s="8"/>
+      <c r="O501" s="8"/>
+    </row>
+    <row r="502" ht="12.75" customHeight="1">
+      <c r="A502" s="34"/>
+      <c r="B502" s="35"/>
+      <c r="C502" s="35"/>
+      <c r="D502" s="35"/>
+      <c r="E502" s="36"/>
+      <c r="F502" s="36"/>
+      <c r="G502" s="36"/>
+      <c r="H502" s="8"/>
+      <c r="I502" s="9"/>
+      <c r="J502" s="22"/>
+      <c r="K502" s="22"/>
+      <c r="L502" s="36"/>
+      <c r="M502" s="8"/>
+      <c r="N502" s="8"/>
+      <c r="O502" s="8"/>
+    </row>
+    <row r="503" ht="12.75" customHeight="1">
+      <c r="A503" s="34"/>
+      <c r="B503" s="35"/>
+      <c r="C503" s="35"/>
+      <c r="D503" s="35"/>
+      <c r="E503" s="36"/>
+      <c r="F503" s="36"/>
+      <c r="G503" s="36"/>
+      <c r="H503" s="8"/>
+      <c r="I503" s="9"/>
+      <c r="J503" s="22"/>
+      <c r="K503" s="22"/>
+      <c r="L503" s="36"/>
+      <c r="M503" s="8"/>
+      <c r="N503" s="8"/>
+      <c r="O503" s="8"/>
+    </row>
+    <row r="504" ht="12.75" customHeight="1">
+      <c r="A504" s="34"/>
+      <c r="B504" s="35"/>
+      <c r="C504" s="35"/>
+      <c r="D504" s="35"/>
+      <c r="E504" s="36"/>
+      <c r="F504" s="36"/>
+      <c r="G504" s="36"/>
+      <c r="H504" s="8"/>
+      <c r="I504" s="9"/>
+      <c r="J504" s="22"/>
+      <c r="K504" s="22"/>
+      <c r="L504" s="36"/>
+      <c r="M504" s="8"/>
+      <c r="N504" s="8"/>
+      <c r="O504" s="8"/>
+    </row>
+    <row r="505" ht="12.75" customHeight="1">
+      <c r="A505" s="34"/>
+      <c r="B505" s="35"/>
+      <c r="C505" s="35"/>
+      <c r="D505" s="35"/>
+      <c r="E505" s="36"/>
+      <c r="F505" s="36"/>
+      <c r="G505" s="36"/>
+      <c r="H505" s="8"/>
+      <c r="I505" s="9"/>
+      <c r="J505" s="22"/>
+      <c r="K505" s="22"/>
+      <c r="L505" s="36"/>
+      <c r="M505" s="8"/>
+      <c r="N505" s="8"/>
+      <c r="O505" s="8"/>
+    </row>
+    <row r="506" ht="12.75" customHeight="1">
+      <c r="A506" s="34"/>
+      <c r="B506" s="35"/>
+      <c r="C506" s="35"/>
+      <c r="D506" s="35"/>
+      <c r="E506" s="36"/>
+      <c r="F506" s="36"/>
+      <c r="G506" s="36"/>
+      <c r="H506" s="8"/>
+      <c r="I506" s="9"/>
+      <c r="J506" s="22"/>
+      <c r="K506" s="22"/>
+      <c r="L506" s="36"/>
+      <c r="M506" s="8"/>
+      <c r="N506" s="8"/>
+      <c r="O506" s="8"/>
+    </row>
+    <row r="507" ht="12.75" customHeight="1">
+      <c r="A507" s="34"/>
+      <c r="B507" s="35"/>
+      <c r="C507" s="35"/>
+      <c r="D507" s="35"/>
+      <c r="E507" s="36"/>
+      <c r="F507" s="36"/>
+      <c r="G507" s="36"/>
+      <c r="H507" s="8"/>
+      <c r="I507" s="9"/>
+      <c r="J507" s="22"/>
+      <c r="K507" s="22"/>
+      <c r="L507" s="36"/>
+      <c r="M507" s="8"/>
+      <c r="N507" s="8"/>
+      <c r="O507" s="8"/>
+    </row>
+    <row r="508" ht="12.75" customHeight="1">
+      <c r="A508" s="34"/>
+      <c r="B508" s="35"/>
+      <c r="C508" s="35"/>
+      <c r="D508" s="35"/>
+      <c r="E508" s="36"/>
+      <c r="F508" s="36"/>
+      <c r="G508" s="36"/>
+      <c r="H508" s="8"/>
+      <c r="I508" s="9"/>
+      <c r="J508" s="22"/>
+      <c r="K508" s="22"/>
+      <c r="L508" s="36"/>
+      <c r="M508" s="8"/>
+      <c r="N508" s="8"/>
+      <c r="O508" s="8"/>
+    </row>
+    <row r="509" ht="12.75" customHeight="1">
+      <c r="A509" s="34"/>
+      <c r="B509" s="35"/>
+      <c r="C509" s="35"/>
+      <c r="D509" s="35"/>
+      <c r="E509" s="36"/>
+      <c r="F509" s="36"/>
+      <c r="G509" s="36"/>
+      <c r="H509" s="8"/>
+      <c r="I509" s="9"/>
+      <c r="J509" s="22"/>
+      <c r="K509" s="22"/>
+      <c r="L509" s="36"/>
+      <c r="M509" s="8"/>
+      <c r="N509" s="8"/>
+      <c r="O509" s="8"/>
+    </row>
+    <row r="510" ht="12.75" customHeight="1">
+      <c r="A510" s="34"/>
+      <c r="B510" s="35"/>
+      <c r="C510" s="35"/>
+      <c r="D510" s="35"/>
+      <c r="E510" s="36"/>
+      <c r="F510" s="36"/>
+      <c r="G510" s="36"/>
+      <c r="H510" s="8"/>
+      <c r="I510" s="9"/>
+      <c r="J510" s="22"/>
+      <c r="K510" s="22"/>
+      <c r="L510" s="36"/>
+      <c r="M510" s="8"/>
+      <c r="N510" s="8"/>
+      <c r="O510" s="8"/>
+    </row>
+    <row r="511" ht="12.75" customHeight="1">
+      <c r="A511" s="34"/>
+      <c r="B511" s="35"/>
+      <c r="C511" s="35"/>
+      <c r="D511" s="35"/>
+      <c r="E511" s="36"/>
+      <c r="F511" s="36"/>
+      <c r="G511" s="36"/>
+      <c r="H511" s="8"/>
+      <c r="I511" s="9"/>
+      <c r="J511" s="22"/>
+      <c r="K511" s="22"/>
+      <c r="L511" s="36"/>
+      <c r="M511" s="8"/>
+      <c r="N511" s="8"/>
+      <c r="O511" s="8"/>
+    </row>
+    <row r="512" ht="12.75" customHeight="1">
+      <c r="A512" s="34"/>
+      <c r="B512" s="35"/>
+      <c r="C512" s="35"/>
+      <c r="D512" s="35"/>
+      <c r="E512" s="36"/>
+      <c r="F512" s="36"/>
+      <c r="G512" s="36"/>
+      <c r="H512" s="8"/>
+      <c r="I512" s="9"/>
+      <c r="J512" s="22"/>
+      <c r="K512" s="22"/>
+      <c r="L512" s="36"/>
+      <c r="M512" s="8"/>
+      <c r="N512" s="8"/>
+      <c r="O512" s="8"/>
+    </row>
+    <row r="513" ht="12.75" customHeight="1">
+      <c r="A513" s="34"/>
+      <c r="B513" s="35"/>
+      <c r="C513" s="35"/>
+      <c r="D513" s="35"/>
+      <c r="E513" s="36"/>
+      <c r="F513" s="36"/>
+      <c r="G513" s="36"/>
+      <c r="H513" s="8"/>
+      <c r="I513" s="9"/>
+      <c r="J513" s="22"/>
+      <c r="K513" s="22"/>
+      <c r="L513" s="36"/>
+      <c r="M513" s="8"/>
+      <c r="N513" s="8"/>
+      <c r="O513" s="8"/>
+    </row>
+    <row r="514" ht="12.75" customHeight="1">
+      <c r="A514" s="34"/>
+      <c r="B514" s="35"/>
+      <c r="C514" s="35"/>
+      <c r="D514" s="35"/>
+      <c r="E514" s="36"/>
+      <c r="F514" s="36"/>
+      <c r="G514" s="36"/>
+      <c r="H514" s="8"/>
+      <c r="I514" s="9"/>
+      <c r="J514" s="22"/>
+      <c r="K514" s="22"/>
+      <c r="L514" s="36"/>
+      <c r="M514" s="8"/>
+      <c r="N514" s="8"/>
+      <c r="O514" s="8"/>
+    </row>
+    <row r="515" ht="12.75" customHeight="1">
+      <c r="A515" s="34"/>
+      <c r="B515" s="35"/>
+      <c r="C515" s="35"/>
+      <c r="D515" s="35"/>
+      <c r="E515" s="36"/>
+      <c r="F515" s="36"/>
+      <c r="G515" s="36"/>
+      <c r="H515" s="8"/>
+      <c r="I515" s="9"/>
+      <c r="J515" s="22"/>
+      <c r="K515" s="22"/>
+      <c r="L515" s="36"/>
+      <c r="M515" s="8"/>
+      <c r="N515" s="8"/>
+      <c r="O515" s="8"/>
+    </row>
+    <row r="516" ht="12.75" customHeight="1">
+      <c r="A516" s="34"/>
+      <c r="B516" s="35"/>
+      <c r="C516" s="35"/>
+      <c r="D516" s="35"/>
+      <c r="E516" s="36"/>
+      <c r="F516" s="36"/>
+      <c r="G516" s="36"/>
+      <c r="H516" s="8"/>
+      <c r="I516" s="9"/>
+      <c r="J516" s="22"/>
+      <c r="K516" s="22"/>
+      <c r="L516" s="36"/>
+      <c r="M516" s="8"/>
+      <c r="N516" s="8"/>
+      <c r="O516" s="8"/>
+    </row>
+    <row r="517" ht="12.75" customHeight="1">
+      <c r="A517" s="34"/>
+      <c r="B517" s="35"/>
+      <c r="C517" s="35"/>
+      <c r="D517" s="35"/>
+      <c r="E517" s="36"/>
+      <c r="F517" s="36"/>
+      <c r="G517" s="36"/>
+      <c r="H517" s="8"/>
+      <c r="I517" s="9"/>
+      <c r="J517" s="22"/>
+      <c r="K517" s="22"/>
+      <c r="L517" s="36"/>
+      <c r="M517" s="8"/>
+      <c r="N517" s="8"/>
+      <c r="O517" s="8"/>
+    </row>
+    <row r="518" ht="12.75" customHeight="1">
+      <c r="A518" s="34"/>
+      <c r="B518" s="35"/>
+      <c r="C518" s="35"/>
+      <c r="D518" s="35"/>
+      <c r="E518" s="36"/>
+      <c r="F518" s="36"/>
+      <c r="G518" s="36"/>
+      <c r="H518" s="8"/>
+      <c r="I518" s="9"/>
+      <c r="J518" s="22"/>
+      <c r="K518" s="22"/>
+      <c r="L518" s="36"/>
+      <c r="M518" s="8"/>
+      <c r="N518" s="8"/>
+      <c r="O518" s="8"/>
+    </row>
+    <row r="519" ht="12.75" customHeight="1">
+      <c r="A519" s="34"/>
+      <c r="B519" s="35"/>
+      <c r="C519" s="35"/>
+      <c r="D519" s="35"/>
+      <c r="E519" s="36"/>
+      <c r="F519" s="36"/>
+      <c r="G519" s="36"/>
+      <c r="H519" s="8"/>
+      <c r="I519" s="9"/>
+      <c r="J519" s="22"/>
+      <c r="K519" s="22"/>
+      <c r="L519" s="36"/>
+      <c r="M519" s="8"/>
+      <c r="N519" s="8"/>
+      <c r="O519" s="8"/>
+    </row>
+    <row r="520" ht="12.75" customHeight="1">
+      <c r="A520" s="34"/>
+      <c r="B520" s="35"/>
+      <c r="C520" s="35"/>
+      <c r="D520" s="35"/>
+      <c r="E520" s="36"/>
+      <c r="F520" s="36"/>
+      <c r="G520" s="36"/>
+      <c r="H520" s="8"/>
+      <c r="I520" s="9"/>
+      <c r="J520" s="22"/>
+      <c r="K520" s="22"/>
+      <c r="L520" s="36"/>
+      <c r="M520" s="8"/>
+      <c r="N520" s="8"/>
+      <c r="O520" s="8"/>
+    </row>
+    <row r="521" ht="12.75" customHeight="1">
+      <c r="A521" s="34"/>
+      <c r="B521" s="35"/>
+      <c r="C521" s="35"/>
+      <c r="D521" s="35"/>
+      <c r="E521" s="36"/>
+      <c r="F521" s="36"/>
+      <c r="G521" s="36"/>
+      <c r="H521" s="8"/>
+      <c r="I521" s="9"/>
+      <c r="J521" s="22"/>
+      <c r="K521" s="22"/>
+      <c r="L521" s="36"/>
+      <c r="M521" s="8"/>
+      <c r="N521" s="8"/>
+      <c r="O521" s="8"/>
+    </row>
+    <row r="522" ht="12.75" customHeight="1">
+      <c r="A522" s="34"/>
+      <c r="B522" s="35"/>
+      <c r="C522" s="35"/>
+      <c r="D522" s="35"/>
+      <c r="E522" s="36"/>
+      <c r="F522" s="36"/>
+      <c r="G522" s="36"/>
+      <c r="H522" s="8"/>
+      <c r="I522" s="9"/>
+      <c r="J522" s="22"/>
+      <c r="K522" s="22"/>
+      <c r="L522" s="36"/>
+      <c r="M522" s="8"/>
+      <c r="N522" s="8"/>
+      <c r="O522" s="8"/>
+    </row>
+    <row r="523" ht="12.75" customHeight="1">
+      <c r="A523" s="34"/>
+      <c r="B523" s="35"/>
+      <c r="C523" s="35"/>
+      <c r="D523" s="35"/>
+      <c r="E523" s="36"/>
+      <c r="F523" s="36"/>
+      <c r="G523" s="36"/>
+      <c r="H523" s="8"/>
+      <c r="I523" s="9"/>
+      <c r="J523" s="22"/>
+      <c r="K523" s="22"/>
+      <c r="L523" s="36"/>
+      <c r="M523" s="8"/>
+      <c r="N523" s="8"/>
+      <c r="O523" s="8"/>
+    </row>
+    <row r="524" ht="12.75" customHeight="1">
+      <c r="A524" s="34"/>
+      <c r="B524" s="35"/>
+      <c r="C524" s="35"/>
+      <c r="D524" s="35"/>
+      <c r="E524" s="36"/>
+      <c r="F524" s="36"/>
+      <c r="G524" s="36"/>
+      <c r="H524" s="8"/>
+      <c r="I524" s="9"/>
+      <c r="J524" s="22"/>
+      <c r="K524" s="22"/>
+      <c r="L524" s="36"/>
+      <c r="M524" s="8"/>
+      <c r="N524" s="8"/>
+      <c r="O524" s="8"/>
+    </row>
+    <row r="525" ht="12.75" customHeight="1">
+      <c r="A525" s="34"/>
+      <c r="B525" s="35"/>
+      <c r="C525" s="35"/>
+      <c r="D525" s="35"/>
+      <c r="E525" s="36"/>
+      <c r="F525" s="36"/>
+      <c r="G525" s="36"/>
+      <c r="H525" s="8"/>
+      <c r="I525" s="9"/>
+      <c r="J525" s="22"/>
+      <c r="K525" s="22"/>
+      <c r="L525" s="36"/>
+      <c r="M525" s="8"/>
+      <c r="N525" s="8"/>
+      <c r="O525" s="8"/>
+    </row>
+    <row r="526" ht="12.75" customHeight="1">
+      <c r="A526" s="34"/>
+      <c r="B526" s="35"/>
+      <c r="C526" s="35"/>
+      <c r="D526" s="35"/>
+      <c r="E526" s="36"/>
+      <c r="F526" s="36"/>
+      <c r="G526" s="36"/>
+      <c r="H526" s="8"/>
+      <c r="I526" s="9"/>
+      <c r="J526" s="22"/>
+      <c r="K526" s="22"/>
+      <c r="L526" s="36"/>
+      <c r="M526" s="8"/>
+      <c r="N526" s="8"/>
+      <c r="O526" s="8"/>
+    </row>
+    <row r="527" ht="12.75" customHeight="1">
+      <c r="A527" s="34"/>
+      <c r="B527" s="35"/>
+      <c r="C527" s="35"/>
+      <c r="D527" s="35"/>
+      <c r="E527" s="36"/>
+      <c r="F527" s="36"/>
+      <c r="G527" s="36"/>
+      <c r="H527" s="8"/>
+      <c r="I527" s="9"/>
+      <c r="J527" s="22"/>
+      <c r="K527" s="22"/>
+      <c r="L527" s="36"/>
+      <c r="M527" s="8"/>
+      <c r="N527" s="8"/>
+      <c r="O527" s="8"/>
+    </row>
+    <row r="528" ht="12.75" customHeight="1">
+      <c r="A528" s="34"/>
+      <c r="B528" s="35"/>
+      <c r="C528" s="35"/>
+      <c r="D528" s="35"/>
+      <c r="E528" s="36"/>
+      <c r="F528" s="36"/>
+      <c r="G528" s="36"/>
+      <c r="H528" s="8"/>
+      <c r="I528" s="9"/>
+      <c r="J528" s="22"/>
+      <c r="K528" s="22"/>
+      <c r="L528" s="36"/>
+      <c r="M528" s="8"/>
+      <c r="N528" s="8"/>
+      <c r="O528" s="8"/>
+    </row>
+    <row r="529" ht="12.75" customHeight="1">
+      <c r="A529" s="34"/>
+      <c r="B529" s="35"/>
+      <c r="C529" s="35"/>
+      <c r="D529" s="35"/>
+      <c r="E529" s="36"/>
+      <c r="F529" s="36"/>
+      <c r="G529" s="36"/>
+      <c r="H529" s="8"/>
+      <c r="I529" s="9"/>
+      <c r="J529" s="22"/>
+      <c r="K529" s="22"/>
+      <c r="L529" s="36"/>
+      <c r="M529" s="8"/>
+      <c r="N529" s="8"/>
+      <c r="O529" s="8"/>
+    </row>
+    <row r="530" ht="12.75" customHeight="1">
+      <c r="A530" s="34"/>
+      <c r="B530" s="35"/>
+      <c r="C530" s="35"/>
+      <c r="D530" s="35"/>
+      <c r="E530" s="36"/>
+      <c r="F530" s="36"/>
+      <c r="G530" s="36"/>
+      <c r="H530" s="8"/>
+      <c r="I530" s="9"/>
+      <c r="J530" s="22"/>
+      <c r="K530" s="22"/>
+      <c r="L530" s="36"/>
+      <c r="M530" s="8"/>
+      <c r="N530" s="8"/>
+      <c r="O530" s="8"/>
+    </row>
+    <row r="531" ht="12.75" customHeight="1">
+      <c r="A531" s="34"/>
+      <c r="B531" s="35"/>
+      <c r="C531" s="35"/>
+      <c r="D531" s="35"/>
+      <c r="E531" s="36"/>
+      <c r="F531" s="36"/>
+      <c r="G531" s="36"/>
+      <c r="H531" s="8"/>
+      <c r="I531" s="9"/>
+      <c r="J531" s="22"/>
+      <c r="K531" s="22"/>
+      <c r="L531" s="36"/>
+      <c r="M531" s="8"/>
+      <c r="N531" s="8"/>
+      <c r="O531" s="8"/>
+    </row>
+    <row r="532" ht="12.75" customHeight="1">
+      <c r="A532" s="34"/>
+      <c r="B532" s="35"/>
+      <c r="C532" s="35"/>
+      <c r="D532" s="35"/>
+      <c r="E532" s="36"/>
+      <c r="F532" s="36"/>
+      <c r="G532" s="36"/>
+      <c r="H532" s="8"/>
+      <c r="I532" s="9"/>
+      <c r="J532" s="22"/>
+      <c r="K532" s="22"/>
+      <c r="L532" s="36"/>
+      <c r="M532" s="8"/>
+      <c r="N532" s="8"/>
+      <c r="O532" s="8"/>
+    </row>
+    <row r="533" ht="12.75" customHeight="1">
+      <c r="A533" s="34"/>
+      <c r="B533" s="35"/>
+      <c r="C533" s="35"/>
+      <c r="D533" s="35"/>
+      <c r="E533" s="36"/>
+      <c r="F533" s="36"/>
+      <c r="G533" s="36"/>
+      <c r="H533" s="8"/>
+      <c r="I533" s="9"/>
+      <c r="J533" s="22"/>
+      <c r="K533" s="22"/>
+      <c r="L533" s="36"/>
+      <c r="M533" s="8"/>
+      <c r="N533" s="8"/>
+      <c r="O533" s="8"/>
+    </row>
+    <row r="534" ht="12.75" customHeight="1">
+      <c r="A534" s="34"/>
+      <c r="B534" s="35"/>
+      <c r="C534" s="35"/>
+      <c r="D534" s="35"/>
+      <c r="E534" s="36"/>
+      <c r="F534" s="36"/>
+      <c r="G534" s="36"/>
+      <c r="H534" s="8"/>
+      <c r="I534" s="9"/>
+      <c r="J534" s="22"/>
+      <c r="K534" s="22"/>
+      <c r="L534" s="36"/>
+      <c r="M534" s="8"/>
+      <c r="N534" s="8"/>
+      <c r="O534" s="8"/>
+    </row>
+    <row r="535" ht="12.75" customHeight="1">
+      <c r="A535" s="34"/>
+      <c r="B535" s="35"/>
+      <c r="C535" s="35"/>
+      <c r="D535" s="35"/>
+      <c r="E535" s="36"/>
+      <c r="F535" s="36"/>
+      <c r="G535" s="36"/>
+      <c r="H535" s="8"/>
+      <c r="I535" s="9"/>
+      <c r="J535" s="22"/>
+      <c r="K535" s="22"/>
+      <c r="L535" s="36"/>
+      <c r="M535" s="8"/>
+      <c r="N535" s="8"/>
+      <c r="O535" s="8"/>
+    </row>
+    <row r="536" ht="12.75" customHeight="1">
+      <c r="A536" s="34"/>
+      <c r="B536" s="35"/>
+      <c r="C536" s="35"/>
+      <c r="D536" s="35"/>
+      <c r="E536" s="36"/>
+      <c r="F536" s="36"/>
+      <c r="G536" s="36"/>
+      <c r="H536" s="8"/>
+      <c r="I536" s="9"/>
+      <c r="J536" s="22"/>
+      <c r="K536" s="22"/>
+      <c r="L536" s="36"/>
+      <c r="M536" s="8"/>
+      <c r="N536" s="8"/>
+      <c r="O536" s="8"/>
+    </row>
+    <row r="537" ht="12.75" customHeight="1">
+      <c r="A537" s="34"/>
+      <c r="B537" s="35"/>
+      <c r="C537" s="35"/>
+      <c r="D537" s="35"/>
+      <c r="E537" s="36"/>
+      <c r="F537" s="36"/>
+      <c r="G537" s="36"/>
+      <c r="H537" s="8"/>
+      <c r="I537" s="9"/>
+      <c r="J537" s="22"/>
+      <c r="K537" s="22"/>
+      <c r="L537" s="36"/>
+      <c r="M537" s="8"/>
+      <c r="N537" s="8"/>
+      <c r="O537" s="8"/>
+    </row>
+    <row r="538" ht="12.75" customHeight="1">
+      <c r="A538" s="34"/>
+      <c r="B538" s="35"/>
+      <c r="C538" s="35"/>
+      <c r="D538" s="35"/>
+      <c r="E538" s="36"/>
+      <c r="F538" s="36"/>
+      <c r="G538" s="36"/>
+      <c r="H538" s="8"/>
+      <c r="I538" s="9"/>
+      <c r="J538" s="22"/>
+      <c r="K538" s="22"/>
+      <c r="L538" s="36"/>
+      <c r="M538" s="8"/>
+      <c r="N538" s="8"/>
+      <c r="O538" s="8"/>
+    </row>
+    <row r="539" ht="12.75" customHeight="1">
+      <c r="A539" s="34"/>
+      <c r="B539" s="35"/>
+      <c r="C539" s="35"/>
+      <c r="D539" s="35"/>
+      <c r="E539" s="36"/>
+      <c r="F539" s="36"/>
+      <c r="G539" s="36"/>
+      <c r="H539" s="8"/>
+      <c r="I539" s="9"/>
+      <c r="J539" s="22"/>
+      <c r="K539" s="22"/>
+      <c r="L539" s="36"/>
+      <c r="M539" s="8"/>
+      <c r="N539" s="8"/>
+      <c r="O539" s="8"/>
+    </row>
+    <row r="540" ht="12.75" customHeight="1">
+      <c r="A540" s="34"/>
+      <c r="B540" s="35"/>
+      <c r="C540" s="35"/>
+      <c r="D540" s="35"/>
+      <c r="E540" s="36"/>
+      <c r="F540" s="36"/>
+      <c r="G540" s="36"/>
+      <c r="H540" s="8"/>
+      <c r="I540" s="9"/>
+      <c r="J540" s="22"/>
+      <c r="K540" s="22"/>
+      <c r="L540" s="36"/>
+      <c r="M540" s="8"/>
+      <c r="N540" s="8"/>
+      <c r="O540" s="8"/>
+    </row>
+    <row r="541" ht="12.75" customHeight="1">
+      <c r="A541" s="34"/>
+      <c r="B541" s="35"/>
+      <c r="C541" s="35"/>
+      <c r="D541" s="35"/>
+      <c r="E541" s="36"/>
+      <c r="F541" s="36"/>
+      <c r="G541" s="36"/>
+      <c r="H541" s="8"/>
+      <c r="I541" s="9"/>
+      <c r="J541" s="22"/>
+      <c r="K541" s="22"/>
+      <c r="L541" s="36"/>
+      <c r="M541" s="8"/>
+      <c r="N541" s="8"/>
+      <c r="O541" s="8"/>
+    </row>
+    <row r="542" ht="12.75" customHeight="1">
+      <c r="A542" s="34"/>
+      <c r="B542" s="35"/>
+      <c r="C542" s="35"/>
+      <c r="D542" s="35"/>
+      <c r="E542" s="36"/>
+      <c r="F542" s="36"/>
+      <c r="G542" s="36"/>
+      <c r="H542" s="8"/>
+      <c r="I542" s="9"/>
+      <c r="J542" s="22"/>
+      <c r="K542" s="22"/>
+      <c r="L542" s="36"/>
+      <c r="M542" s="8"/>
+      <c r="N542" s="8"/>
+      <c r="O542" s="8"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -22941,13 +24881,18 @@
     <hyperlink r:id="rId439" ref="I440"/>
     <hyperlink r:id="rId440" ref="I441"/>
     <hyperlink r:id="rId441" ref="I442"/>
+    <hyperlink r:id="rId442" ref="I443"/>
+    <hyperlink r:id="rId443" ref="I444"/>
+    <hyperlink r:id="rId444" ref="I445"/>
+    <hyperlink r:id="rId445" ref="I446"/>
+    <hyperlink r:id="rId446" ref="I447"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup paperSize="9" orientation="portrait"/>
-  <drawing r:id="rId442"/>
+  <drawing r:id="rId447"/>
   <tableParts count="1">
-    <tablePart r:id="rId444"/>
+    <tablePart r:id="rId449"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>